<commit_message>
Primer Parcial con Totales Academia Corregidos
</commit_message>
<xml_diff>
--- a/academias/Administración de Recursos Humanos - Estadisticos 20222.xlsx
+++ b/academias/Administración de Recursos Humanos - Estadisticos 20222.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="29">
   <si>
     <t>Docente</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Mendoza Velazquez Laura Elena</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>ELABORA ESTRATEGIAS PARA REALIZAR LAS ACTIVIDADES DE SU ÁREA</t>
   </si>
   <si>
@@ -77,10 +74,16 @@
     <t>DETERMINA REMUNERACIONES DEL PERSONAL EN SITUACIONES EXTRAORDINARIAS</t>
   </si>
   <si>
+    <t>Totales Docente</t>
+  </si>
+  <si>
     <t>EVALÚA EL DESEMPEÑO DE LA ORGANIZACIÓN UTILIZANDO HERRAMIENTAS DE CALIDAD</t>
   </si>
   <si>
     <t>DISTINGUE LOS DIFERENTES TIPOS DE EMPRESA POR SU GIRO, ÁREAS FUNCIONALES, DOCUMENTACIÓN ADMINISTRATIVA Y RECURSOS</t>
+  </si>
+  <si>
+    <t>Totales Generales</t>
   </si>
   <si>
     <t>2ARHV</t>
@@ -466,7 +469,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="50.7109375" customWidth="1"/>
     <col min="7" max="8" width="9.140625" style="1"/>
     <col min="9" max="9" width="9.140625" style="2"/>
     <col min="11" max="11" width="9.140625" style="1"/>
@@ -512,10 +515,10 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2">
         <v>33</v>
@@ -547,10 +550,10 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3">
         <v>30</v>
@@ -582,10 +585,10 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4">
         <v>36</v>
@@ -617,10 +620,10 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5">
         <v>31</v>
@@ -651,6 +654,9 @@
       <c r="A6" t="s">
         <v>11</v>
       </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
       <c r="D6">
         <v>130</v>
       </c>
@@ -681,10 +687,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7">
         <v>40</v>
@@ -716,10 +722,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D8">
         <v>38</v>
@@ -751,10 +757,10 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D9">
         <v>36</v>
@@ -785,6 +791,9 @@
       <c r="A10" t="s">
         <v>12</v>
       </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
       <c r="D10">
         <v>114</v>
       </c>
@@ -818,7 +827,7 @@
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11">
         <v>30</v>
@@ -850,10 +859,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D12">
         <v>31</v>
@@ -884,6 +893,9 @@
       <c r="A13" t="s">
         <v>13</v>
       </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
       <c r="D13">
         <v>61</v>
       </c>
@@ -917,7 +929,7 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14">
         <v>40</v>
@@ -952,7 +964,7 @@
         <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D15">
         <v>33</v>
@@ -987,7 +999,7 @@
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D16">
         <v>38</v>
@@ -1018,6 +1030,9 @@
       <c r="A17" t="s">
         <v>14</v>
       </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
       <c r="D17">
         <v>111</v>
       </c>
@@ -1044,8 +1059,8 @@
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" t="s">
-        <v>15</v>
+      <c r="B18" t="s">
+        <v>22</v>
       </c>
       <c r="D18">
         <v>416</v>
@@ -1129,10 +1144,10 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2">
         <v>33</v>
@@ -1164,10 +1179,10 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3">
         <v>30</v>
@@ -1199,10 +1214,10 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4">
         <v>36</v>
@@ -1234,10 +1249,10 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5">
         <v>31</v>
@@ -1268,6 +1283,9 @@
       <c r="A6" t="s">
         <v>11</v>
       </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
       <c r="D6">
         <v>130</v>
       </c>
@@ -1298,10 +1316,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7">
         <v>40</v>
@@ -1333,10 +1351,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D8">
         <v>38</v>
@@ -1368,10 +1386,10 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D9">
         <v>36</v>
@@ -1402,6 +1420,9 @@
       <c r="A10" t="s">
         <v>12</v>
       </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
       <c r="D10">
         <v>114</v>
       </c>
@@ -1435,7 +1456,7 @@
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11">
         <v>30</v>
@@ -1467,10 +1488,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D12">
         <v>31</v>
@@ -1501,6 +1522,9 @@
       <c r="A13" t="s">
         <v>13</v>
       </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
       <c r="D13">
         <v>61</v>
       </c>
@@ -1534,7 +1558,7 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14">
         <v>40</v>
@@ -1569,7 +1593,7 @@
         <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D15">
         <v>33</v>
@@ -1604,7 +1628,7 @@
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D16">
         <v>38</v>
@@ -1635,6 +1659,9 @@
       <c r="A17" t="s">
         <v>14</v>
       </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
       <c r="D17">
         <v>111</v>
       </c>
@@ -1661,8 +1688,8 @@
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" t="s">
-        <v>15</v>
+      <c r="B18" t="s">
+        <v>22</v>
       </c>
       <c r="D18">
         <v>416</v>

</xml_diff>